<commit_message>
chore: add data migration and analysis scripts
Swooped import scripts (job descriptions, cover letters, closed dates),
application analysis, content migration, cover letter cleanup, and
updated billing/tracker data.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$K$1</definedName>
@@ -11119,7 +11119,6 @@
       </c>
     </row>
     <row r="332">
-      <c r="A332" t="inlineStr"/>
       <c r="B332" t="inlineStr">
         <is>
           <t>Abacus Insights</t>
@@ -11152,7 +11151,6 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="inlineStr"/>
       <c r="B333" t="inlineStr">
         <is>
           <t>Jobgether</t>
@@ -11185,7 +11183,6 @@
       </c>
     </row>
     <row r="334">
-      <c r="A334" t="inlineStr"/>
       <c r="B334" t="inlineStr">
         <is>
           <t>iVoyant</t>
@@ -11218,7 +11215,6 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" t="inlineStr"/>
       <c r="B335" t="inlineStr">
         <is>
           <t>Jobgether</t>
@@ -11251,7 +11247,6 @@
       </c>
     </row>
     <row r="336">
-      <c r="A336" t="inlineStr"/>
       <c r="B336" t="inlineStr">
         <is>
           <t>Castlight Health</t>
@@ -11284,7 +11279,6 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="inlineStr"/>
       <c r="B337" t="inlineStr">
         <is>
           <t>A Place for Mom</t>
@@ -11317,7 +11311,6 @@
       </c>
     </row>
     <row r="338">
-      <c r="A338" t="inlineStr"/>
       <c r="B338" t="inlineStr">
         <is>
           <t>AutoPylot</t>
@@ -11350,7 +11343,6 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="inlineStr"/>
       <c r="B339" t="inlineStr">
         <is>
           <t>Forward Financing</t>
@@ -11383,7 +11375,6 @@
       </c>
     </row>
     <row r="340">
-      <c r="A340" t="inlineStr"/>
       <c r="B340" t="inlineStr">
         <is>
           <t>Mira Energy Group,</t>
@@ -11416,7 +11407,6 @@
       </c>
     </row>
     <row r="341">
-      <c r="A341" t="inlineStr"/>
       <c r="B341" t="inlineStr">
         <is>
           <t>Motional</t>
@@ -11449,7 +11439,6 @@
       </c>
     </row>
     <row r="342">
-      <c r="A342" t="inlineStr"/>
       <c r="B342" t="inlineStr">
         <is>
           <t>NinjaOne</t>
@@ -11482,7 +11471,6 @@
       </c>
     </row>
     <row r="343">
-      <c r="A343" t="inlineStr"/>
       <c r="B343" t="inlineStr">
         <is>
           <t>Paradigm Health</t>
@@ -11515,7 +11503,6 @@
       </c>
     </row>
     <row r="344">
-      <c r="A344" t="inlineStr"/>
       <c r="B344" t="inlineStr">
         <is>
           <t>Perfecting Peds</t>
@@ -11548,7 +11535,6 @@
       </c>
     </row>
     <row r="345">
-      <c r="A345" t="inlineStr"/>
       <c r="B345" t="inlineStr">
         <is>
           <t>REVEL SEARCH®</t>
@@ -11581,7 +11567,6 @@
       </c>
     </row>
     <row r="346">
-      <c r="A346" t="inlineStr"/>
       <c r="B346" t="inlineStr">
         <is>
           <t>Ventra Health</t>
@@ -11614,7 +11599,6 @@
       </c>
     </row>
     <row r="347">
-      <c r="A347" t="inlineStr"/>
       <c r="B347" t="inlineStr">
         <is>
           <t>Vice President of</t>
@@ -11647,7 +11631,6 @@
       </c>
     </row>
     <row r="348">
-      <c r="A348" t="inlineStr"/>
       <c r="B348" t="inlineStr">
         <is>
           <t>X4 Life Sciences</t>

</xml_diff>

<commit_message>
fix: full pipeline audit — fetch, parse, source, and score all Gmail leads
Ran end-to-end audit of Gmail vs pipeline. Found 14 unfetched emails
and 13 parsed-but-unsourced leads. Fixed all gaps:
- Fetched 14 new emails (UIDs 33-46)
- Sourced all 145 leads (was 57)
- Scored 126 leads, created 60 new application folders
- Fixed DIRECTV rejection (UID 45) misclassified as unresolved
- Fixed Unicode crash in career_search.py (cp1252 encoding)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Applications" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Applications'!$A$1:$K$1</definedName>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K348"/>
+  <dimension ref="A1:K408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11662,6 +11662,1986 @@
         </is>
       </c>
     </row>
+    <row r="349">
+      <c r="A349" t="inlineStr"/>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>VP, Engineering REMOTE</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr"/>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Remote Senior Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr"/>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Senior VP of Software Engineering - REMOTE</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr"/>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Remote Lead Software Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr"/>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>PointClickCare</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Manager Software Engineering</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr"/>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Senior Director of Engineering</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr"/>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Cambium Learning</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>VP, Innovation and Engineering</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr"/>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Freenome</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Vice President, Digital Health</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr"/>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Alimentiv</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Manager, Software Development &amp; Testing</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr"/>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>AlphaPoint</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>VP of Engineering opening</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr"/>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>AMN Healthcare Leadership Solutions | B.E. Smith</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Chief Digital Information Officer</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr"/>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Appspace</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Vice President of Architecture &amp; AI Engineering Transformation</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr"/>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Brightline</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Senior Manager/Director, Engineering</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr"/>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Confidential</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Engineering Manager, AI Capabilities</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr"/>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Crunchafi</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>VP of Engineering</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr"/>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>CSG</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Director of Software Development role</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr"/>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Dandy</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr"/>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Ensemble Health Partners</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>VP, Engineering</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr"/>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Evolent</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Senior Director, Software Engineering</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr"/>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>GE HealthCare</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Senior Director</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr"/>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>GenBio AI</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Vice President of Engineering</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr"/>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Gyga Force</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Software Engineering Manager – SaaS Platform</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr"/>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Hanalytica GmbH</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Software Development Manager</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr"/>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>HiroJet</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr"/>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>James Search</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Vice President of Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr"/>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Remote VP Engineering</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr"/>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Senior Engineering VP - REMOTE</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr"/>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr"/>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Jobgether</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>VP of Software Engineering</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr"/>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Just Appraised</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr"/>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>kadence</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Founding Head of Engineering</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr"/>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Kaufman Rossin</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Chief Information Officer</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr"/>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Ladders</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Senior Manager, Engineering</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr"/>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Lettuce Box,</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Head of Engineering</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr"/>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Madison-Davis,</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr"/>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Meade Engineering,</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Vice President of Engineering</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr"/>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Odyssey Information Services</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Software Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr"/>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Pathfinders Executive Search</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr"/>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Payroll Integrations</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr"/>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Restaurant Brands International</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Vice President, Engineering</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr"/>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Richard Lombart Consulting &amp; The Executive Way</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Chief Technology Innovation Officer</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr"/>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Shutterfly</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Senior Manager, Software Engineering</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr"/>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>SimplePractice</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Senior Manager of Machine Learning, Applied AI</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr"/>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Solution Community</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Head of Engineering (Volunteer)</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr"/>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Spectrum Search</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>CTO / Tech Lead</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr"/>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Stord</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr"/>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Architect role</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr"/>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>TENEX.AI</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Head of Platform Engineering</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr"/>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Senior Manager, Platform Engineering</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr"/>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Thermo Fisher Scientific</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Director, Product Engineering</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr"/>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Thrive Resources</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>VP, Platform Engineering</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr"/>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Torticity</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr"/>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Uneek Global</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Software Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr"/>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>VCU Health</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Associate Vice President, Healthcare Digital Transformation</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr"/>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>WME | William Morris Endeavor</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Head of Engineering</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr"/>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>XYZ Match</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr"/>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>ŌURA</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr"/>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Compass Health Center</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Senior Vice President, Technology &amp; Data Solutions</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr"/>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Relativity</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Manager, Software Engineering</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr"/>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Onebrief</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Engineering Manager, Developer Experience</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Email Pipeline</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Pending Review</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Long Shot</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>Sourced via email pipeline</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>